<commit_message>
Add Pampadu tracking links for 13 offers; show ad marking (erid) on vacancy cards
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015gDLhwgHQJ9auhFtnwdBUw
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -83,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -112,6 +112,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -207,6 +211,11 @@
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <t>Колонки R–Y — служебные, бот их не показывает. Источник: выгрузка офферов Pampadu от 07.10.2026.</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
+        <t>Рекламодатель для маркировки: название и ИНН из карточки оффера Pampadu (например «ООО Яндекс.Еда, ИНН …»). Бот показывает его в строке «Реклама» под вакансией.</t>
       </text>
     </comment>
   </commentList>
@@ -502,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y17"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -530,6 +539,7 @@
     <col width="7" customWidth="1" min="23" max="23"/>
     <col width="30" customWidth="1" min="24" max="24"/>
     <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -658,6 +668,11 @@
           <t>to_verify</t>
         </is>
       </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>advertiser</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -708,7 +723,11 @@
           <t>Паспорт, смартфон</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/7BjQFfpI?erid=CQH36pWzJqVGXC5oLP8WVVNCNqJmbhiUPijGiu4zpwPd7G</t>
+        </is>
+      </c>
       <c r="P2" s="3" t="n">
         <v>1</v>
       </c>
@@ -745,6 +764,7 @@
           <t>Что входит в «активность» (сколько заказов); работает ли в Екб</t>
         </is>
       </c>
+      <c r="Z2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -795,7 +815,11 @@
           <t>Паспорт, смартфон</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/atmfMiR1?erid=2SDnjcXP37s</t>
+        </is>
+      </c>
       <c r="P3" s="3" t="n">
         <v>2</v>
       </c>
@@ -832,6 +856,7 @@
           <t>Какие смены доступны в Екб</t>
         </is>
       </c>
+      <c r="Z3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -882,7 +907,11 @@
           <t>Паспорт; уточнить, нужна ли медкнижка</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/jqrQfjbR?erid=CQH36pWzJqVGXC5oUHvq1FTH2g3oi1KL72bsqkyo9iVXM7</t>
+        </is>
+      </c>
       <c r="P4" s="3" t="n">
         <v>3</v>
       </c>
@@ -915,6 +944,7 @@
           <t>Нужна ли медкнижка; что входит в «активность»</t>
         </is>
       </c>
+      <c r="Z4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -965,7 +995,11 @@
           <t>Паспорт</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/0Hwvv7Yl?erid=Kra23pBTF</t>
+        </is>
+      </c>
       <c r="P5" s="3" t="n">
         <v>4</v>
       </c>
@@ -998,6 +1032,7 @@
           <t>Оплата за валидную заявку — проверить требования к заявке</t>
         </is>
       </c>
+      <c r="Z5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -1048,7 +1083,11 @@
           <t>Паспорт</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/OXxVEOxP?erid=2SDnjbsvvT3</t>
+        </is>
+      </c>
       <c r="P6" s="3" t="n">
         <v>5</v>
       </c>
@@ -1085,6 +1124,7 @@
           <t>Требования к кандидату; нужно ли авто</t>
         </is>
       </c>
+      <c r="Z6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -1135,7 +1175,11 @@
           <t>Паспорт, грамотная речь</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/ocGMbmFE?erid=2SDnjdhc8em</t>
+        </is>
+      </c>
       <c r="P7" s="3" t="n">
         <v>6</v>
       </c>
@@ -1168,6 +1212,7 @@
           <t>Есть ли удалённый формат (тогда remote=1)</t>
         </is>
       </c>
+      <c r="Z7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1218,7 +1263,11 @@
           <t>Паспорт, медкнижка (обычно оформляют при трудоустройстве)</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/yvI1IVFB?erid=2SDnjdu6ZqS</t>
+        </is>
+      </c>
       <c r="P8" s="3" t="n">
         <v>7</v>
       </c>
@@ -1251,6 +1300,7 @@
           <t>Нужна ли медкнижка заранее</t>
         </is>
       </c>
+      <c r="Z8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1301,7 +1351,11 @@
           <t>Компьютер, интернет; для репетиторов — знание предмета</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr"/>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/T9eAPy3s?erid=2SDnjeLCgoN</t>
+        </is>
+      </c>
       <c r="P9" s="3" t="n">
         <v>8</v>
       </c>
@@ -1338,6 +1392,7 @@
           <t>Какие вакансии открыты (репетиторы/менеджеры), требования</t>
         </is>
       </c>
+      <c r="Z9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1421,6 +1476,7 @@
           <t>Требования; что входит в «активность»</t>
         </is>
       </c>
+      <c r="Z10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1471,7 +1527,11 @@
           <t>Паспорт</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/tF4Amn1p?erid=2SDnjcbs16H</t>
+        </is>
+      </c>
       <c r="P11" s="3" t="n">
         <v>10</v>
       </c>
@@ -1508,6 +1568,7 @@
           <t>Какие направления открыты в Екб, есть ли удалёнка</t>
         </is>
       </c>
+      <c r="Z11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1558,7 +1619,11 @@
           <t>Навыки ремонта, свой инструмент</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr"/>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/wxFOcAAz?erid=2SDnjceSYW1</t>
+        </is>
+      </c>
       <c r="P12" s="3" t="n">
         <v>11</v>
       </c>
@@ -1595,6 +1660,7 @@
           <t>Какие специальности принимают</t>
         </is>
       </c>
+      <c r="Z12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1645,7 +1711,11 @@
           <t>Паспорт, смартфон</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr"/>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/4xuC9vhp?erid=2SDnjeL6Zwp</t>
+        </is>
+      </c>
       <c r="P13" s="3" t="n">
         <v>12</v>
       </c>
@@ -1682,6 +1752,7 @@
           <t>В названии «// SMS» — разрешён ли трафик из Telegram. Включить (active=1) после ответа</t>
         </is>
       </c>
+      <c r="Z13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1732,7 +1803,11 @@
           <t>Права категории C (уточнить), стаж</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/sFZC7wSW?erid=CQH36pWzJqVGXC5oTTDpMBk8ei82kpZxV9ZJ1ZC292TAKx</t>
+        </is>
+      </c>
       <c r="P14" s="3" t="n">
         <v>13</v>
       </c>
@@ -1765,6 +1840,7 @@
           <t>Категория прав, минимальный возраст и стаж</t>
         </is>
       </c>
+      <c r="Z14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1815,7 +1891,11 @@
           <t>Паспорт</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr"/>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>https://trk.ppdu.ru/click/u2kZ5X8T?erid=CQH36pWzJqVGXC5oUnPkDCzrr2NGbNEh3prkX12H6fxb5H</t>
+        </is>
+      </c>
       <c r="P15" s="3" t="n">
         <v>14</v>
       </c>
@@ -1852,6 +1932,7 @@
           <t>Условия вахты, куда ехать, жильё</t>
         </is>
       </c>
+      <c r="Z15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1933,6 +2014,7 @@
           <t>Честно указать: без фиксированной оплаты</t>
         </is>
       </c>
+      <c r="Z16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -2014,6 +2096,7 @@
           <t>Честно указать: без фиксированной оплаты</t>
         </is>
       </c>
+      <c r="Z17" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Y17"/>
@@ -2033,7 +2116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2048,7 +2131,7 @@
       </c>
       <c r="B1" s="8" t="inlineStr">
         <is>
-          <t>Жёлтые ячейки на листе jobs: pay_text (текст о доходе) и link (партнёрская ссылка). Без ссылки вакансия не будет работать.</t>
+          <t>Жёлтые ячейки на листе jobs: pay_text (текст о доходе), link (партнёрская ссылка) и advertiser (рекламодатель для маркировки). Без ссылки вакансия не показывается.</t>
         </is>
       </c>
     </row>
@@ -2201,28 +2284,40 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>advertiser</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Рекламодатель для маркировки (название, ИНН) из карточки оффера. Показывается в строке «Реклама … erid» под вакансией</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>payout_rub … to_verify</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Служебные поля для тебя, пользователю не показываются</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr"/>
-      <c r="B16" s="8" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr"/>
+      <c r="B17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Исключены из базы</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>1617, 2381, 2666 — Яндекс.Еда для КЗ/УЗ/Боливии; 1372 — Альфа-Банк для малых городов; 1034 — найм affiliate-менеджера в Pampadu</t>
         </is>

</xml_diff>

<commit_message>
Fill Ekaterinburg income for courier offer 2304
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015gDLhwgHQJ9auhFtnwdBUw
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -216,6 +216,11 @@
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Рекламодатель для маркировки: название и ИНН из карточки оффера Pampadu (например «ООО Яндекс.Еда, ИНН …»). Бот показывает его в строке «Реклама» под вакансией.</t>
+      </text>
+    </comment>
+    <comment ref="M2" authorId="0" shapeId="0">
+      <text>
+        <t>Источник: таблица дохода курьеров по городам, строка «Екатеринбург» (доход в час: авто 894, пеший 582, вело 715; в месяц: 200 160 / 130 320 / 160 200). https://docs.google.com/spreadsheets/d/1jePQrqubaTVlohVZ4126fqfTKRFLaRe0yIWcPpKkEHY Данные получены 09.10.2026, обновлять раз в месяц.</t>
       </text>
     </comment>
   </commentList>
@@ -714,10 +719,14 @@
       <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Доставка заказов пешком, на велосипеде или самокате. Смены выбираешь сам в приложении.</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr"/>
+          <t>Доставка заказов пешком, на велосипеде, самокате или своём авто. Смены выбираешь сам в приложении.</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>В среднем по Екатеринбургу: пешком ≈ 580 ₽/час, на велосипеде ≈ 715 ₽/час, на авто ≈ 890 ₽/час. Итог зависит от числа заказов и часов.</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Паспорт, смартфон</t>

</xml_diff>

<commit_message>
Apply Pampadu offer conditions: requirements, income, advertisers; enable only offers allowing chatbots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015gDLhwgHQJ9auhFtnwdBUw
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -221,6 +221,66 @@
     <comment ref="M2" authorId="0" shapeId="0">
       <text>
         <t>Источник: таблица дохода курьеров по городам, строка «Екатеринбург» (доход в час: авто 894, пеший 582, вело 715; в месяц: 200 160 / 130 320 / 160 200). https://docs.google.com/spreadsheets/d/1jePQrqubaTVlohVZ4126fqfTKRFLaRe0yIWcPpKkEHY Данные получены 09.10.2026, обновлять раз в месяц.</t>
+      </text>
+    </comment>
+    <comment ref="X2" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/kur-er-v-yandeks-eda-yandeks-lavka-rf-rb/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X3" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/yandeks-smena/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X4" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/kladovschik-yandeks-lavka/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X5" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/kur-er-operator-sklada-ozon/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X7" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/operator-call-tsentra-mts/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X8" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/povar-kassir-v-burger-king/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X9" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/tetrika-vakansii/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X11" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/t-bank-rabota-v-t-banke-massovyi-nabor/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X12" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/servis-ruki/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X13" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/kuper-ex-sbermarket-vakansii/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X14" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/voditel-gruzovogo-avtomobilya-yandeks-dostavka/ (проверено 09.10.2026)</t>
+      </text>
+    </comment>
+    <comment ref="X15" authorId="0" shapeId="0">
+      <text>
+        <t>Условия: https://pampadu.ru/affiliate-program/hr-offers/yandeks-market-kladovschiki-vakhta/ (проверено 09.10.2026)</t>
       </text>
     </comment>
   </commentList>
@@ -685,7 +745,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Курьер Яндекс.Еды / Яндекс Лавки</t>
+          <t>Курьер-партнёр сервиса Яндекс Еда / Яндекс Лавка</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -719,7 +779,7 @@
       <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Доставка заказов пешком, на велосипеде, самокате или своём авто. Смены выбираешь сам в приложении.</t>
+          <t>Доставка заказов пешком, на велосипеде, самокате или своём авто. Слоты выбираешь сам в приложении, заказы есть круглосуточно.</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -729,7 +789,7 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Паспорт, смартфон</t>
+          <t>Паспорт; смартфон Android 8+ или iOS 16.5+; медкнижка (оформляется самостоятельно, 1 500–2 000 ₽; самозанятые могут начать без неё)</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -770,7 +830,7 @@
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
-          <t>Что входит в «активность» (сколько заказов); работает ли в Екб</t>
+          <t>Есть ли Екатеринбург в гео (раздел «Баннеры»). Конверсия = 5 заказов за 14 дней. Чат-боты разрешены; нельзя крупные TG-каналы 50k+. В рекламе писать «партнёр сервиса», без слов про трудоустройство</t>
         </is>
       </c>
       <c r="Z2" s="10" t="n"/>
@@ -781,7 +841,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Подработка сменами — Яндекс Смена</t>
+          <t>Задания в магазинах и на складах — партнёр сервиса Яндекс Смена</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -815,13 +875,17 @@
       <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Разовые смены на складах и в магазинах через приложение. Берёшь смену, когда удобно.</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr"/>
+          <t>Задания в торговых точках через приложение: выбираешь удобное время и приходишь к назначенному часу.</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Доход до 3 400 ₽ в день.</t>
+        </is>
+      </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Паспорт, смартфон</t>
+          <t>Паспорт; медкнижка (можно оформить); статус самозанятого (можно оформить)</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
@@ -833,7 +897,7 @@
         <v>2</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R3" s="5" t="n">
         <v>1260</v>
@@ -862,7 +926,7 @@
       </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
-          <t>Какие смены доступны в Екб</t>
+          <t>ВЫКЛЮЧЕН: чат-боты в разрешённых источниках не указаны — спросить менеджера. Гео не подтверждено. В рекламе нельзя слова «работа», «подработка», «зарплата», нельзя возраст и гражданство</t>
         </is>
       </c>
       <c r="Z3" s="10" t="n"/>
@@ -873,7 +937,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Кладовщик в Яндекс Лавке</t>
+          <t>Кладовщик-сборщик у партнёра сервиса Яндекс Лавка</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -894,11 +958,11 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2/2,5/2,night</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="J4" s="3" t="n">
@@ -907,13 +971,17 @@
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Сборка заказов и приёмка товара на складе-магазине рядом с домом.</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr"/>
+          <t>Сборка и упаковка заказов, приёмка и выкладка товара. Официальное оформление, график 5/2 по 8 часов: утро 7:00–16:00 или вечер 15:00–00:00.</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Официальное оформление по ТК, выплаты 2 раза в месяц, ДМС, обеды за 95 ₽ в дарксторах с кухней.</t>
+        </is>
+      </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Паспорт; уточнить, нужна ли медкнижка</t>
+          <t>Паспорт; медкнижку оформляют бесплатно</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
@@ -950,7 +1018,7 @@
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Нужна ли медкнижка; что входит в «активность»</t>
+          <t>Екатеринбург в гео есть. Конверсия = 40 часов за 14 дней. Чат-боты разрешены. В рекламе — «Партнер сервиса Яндекс.Лавка»</t>
         </is>
       </c>
       <c r="Z4" s="10" t="n"/>
@@ -995,7 +1063,7 @@
       <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Доставка или работа на складе Ozon: сборка, упаковка, сортировка.</t>
+          <t>Доставка заказов или работа на складе Ozon: сборка, упаковка, сортировка. График подбирается индивидуально, фирменная форма.</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr"/>
@@ -1038,7 +1106,7 @@
       </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
-          <t>Оплата за валидную заявку — проверить требования к заявке</t>
+          <t>Есть ли Екатеринбург в гео (раздел «Промоматериалы»). Что считается валидной заявкой. Чат-боты разрешены. В рекламе НЕЛЬЗЯ указывать пол, возраст, гражданство, наличие авто</t>
         </is>
       </c>
       <c r="Z5" s="10" t="n"/>
@@ -1089,7 +1157,7 @@
       <c r="M6" s="4" t="inlineStr"/>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Паспорт</t>
+          <t>Паспорт; отсутствие судимости</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
@@ -1101,7 +1169,7 @@
         <v>5</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" s="5" t="n">
         <v>5163.93</v>
@@ -1130,7 +1198,7 @@
       </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>Требования к кандидату; нужно ли авто</t>
+          <t>ВЫКЛЮЧЕН: чат-боты не указаны — спросить менеджера. Гео в «Промоматериалах». Возраст 18–40</t>
         </is>
       </c>
       <c r="Z6" s="10" t="n"/>
@@ -1170,18 +1238,22 @@
         </is>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Консультирование клиентов по телефону. Обучение за счёт компании.</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr"/>
+          <t>Консультирование клиентов МТС по телефону, удалённо. Гибкий график, подбирается индивидуально.</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>ДМС с первого месяца, бесплатная мобильная связь.</t>
+        </is>
+      </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>Паспорт, грамотная речь</t>
+          <t>Паспорт РФ; для молодых людей — приписное или военный билет</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
@@ -1193,7 +1265,7 @@
         <v>6</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R7" s="5" t="n">
         <v>6060.6</v>
@@ -1218,10 +1290,14 @@
       </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>Есть ли удалённый формат (тогда remote=1)</t>
-        </is>
-      </c>
-      <c r="Z7" s="10" t="n"/>
+          <t>ВЫКЛЮЧЕН: чат-боты не указаны (рассылки в мессенджерах и посты разрешены) — спросить менеджера. Гео в «Баннерах»</t>
+        </is>
+      </c>
+      <c r="Z7" s="8" t="inlineStr">
+        <is>
+          <t>ПАО «МТС», ИНН 7740000076</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1263,13 +1339,17 @@
       <c r="K8" s="3" t="inlineStr"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Работа на кухне и кассе ресторана. Гибкий график под учёбу.</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr"/>
+          <t>Работа на кухне и кассе ресторана, можно без опыта. Гибкий график, официальное оформление.</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Официальное оформление, зарплата на карту, премии, бесплатное питание и форма.</t>
+        </is>
+      </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>Паспорт, медкнижка (обычно оформляют при трудоустройстве)</t>
+          <t>Паспорт, свободный русский язык; медкнижку оформляют бесплатно</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
@@ -1306,10 +1386,14 @@
       </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t>Нужна ли медкнижка заранее</t>
-        </is>
-      </c>
-      <c r="Z8" s="10" t="n"/>
+          <t>Есть ли Екатеринбург в гео (раздел «Баннеры»). Чат-боты разрешены</t>
+        </is>
+      </c>
+      <c r="Z8" s="8" t="inlineStr">
+        <is>
+          <t>ООО «БУРГЕР РУС», ИНН 7719723690</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1369,7 +1453,7 @@
         <v>8</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R9" s="5" t="n">
         <v>4015.9</v>
@@ -1398,7 +1482,7 @@
       </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t>Какие вакансии открыты (репетиторы/менеджеры), требования</t>
+          <t>ВЫКЛЮЧЕН: нужны репетиторы со стажем преподавания от 6 лет — не наша аудитория 18–25</t>
         </is>
       </c>
       <c r="Z9" s="10" t="n"/>
@@ -1545,7 +1629,7 @@
         <v>10</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R11" s="5" t="n">
         <v>7350</v>
@@ -1574,7 +1658,7 @@
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t>Какие направления открыты в Екб, есть ли удалёнка</t>
+          <t>ВЫКЛЮЧЕН: чат-боты и рассылки только по согласованию с менеджером. Вакансии и гео — в «Баннерах». Возраст 18–55, гражданство РФ</t>
         </is>
       </c>
       <c r="Z11" s="10" t="n"/>
@@ -1637,7 +1721,7 @@
         <v>11</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R12" s="5" t="n">
         <v>5600</v>
@@ -1666,10 +1750,14 @@
       </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>Какие специальности принимают</t>
-        </is>
-      </c>
-      <c r="Z12" s="10" t="n"/>
+          <t>ВЫКЛЮЧЕН: гео только Москва, мужчины с опытом установки дверей/сборки кухонь от 1 года</t>
+        </is>
+      </c>
+      <c r="Z12" s="8" t="inlineStr">
+        <is>
+          <t>ООО «СЕРВИС ПРО.РЕМОНТ», ИНН 7714418406</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1758,10 +1846,14 @@
       </c>
       <c r="Y13" s="3" t="inlineStr">
         <is>
-          <t>В названии «// SMS» — разрешён ли трафик из Telegram. Включить (active=1) после ответа</t>
-        </is>
-      </c>
-      <c r="Z13" s="10" t="n"/>
+          <t>ВЫКЛЮЧЕН: оффер приостановлен Pampadu. SMS запрещены, чат-боты разрешены — включить, когда оффер возобновят</t>
+        </is>
+      </c>
+      <c r="Z13" s="8" t="inlineStr">
+        <is>
+          <t>ООО «ИНСТАМАРТ СЕРВИС», ИНН 9705118142</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1769,7 +1861,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Водитель грузового авто — Яндекс.Доставка</t>
+          <t>Водитель-партнёр сервиса Яндекс Доставка (грузовой фургон)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1784,10 +1876,10 @@
         <v>1</v>
       </c>
       <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3" t="n">
         <v>1</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>40</v>
@@ -1803,13 +1895,13 @@
       <c r="K14" s="3" t="inlineStr"/>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>Доставка грузов на автомобиле компании или партнёра.</t>
+          <t>Доставка грузов на своём фургоне или на арендованном через автопарк. Можно как основной доход или заказы по городу в свободное время.</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>Права категории C (уточнить), стаж</t>
+          <t>Права категории B или C, СТС; фургон (тент, будка или цельнометаллический), кузов от 190×100×90 см, не старше 2002 г.</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -1846,7 +1938,7 @@
       </c>
       <c r="Y14" s="3" t="inlineStr">
         <is>
-          <t>Категория прав, минимальный возраст и стаж</t>
+          <t>Екатеринбург в гео есть. Конверсия = 5 заказов за 30 дней. Чат-боты разрешены. Без слов про трудоустройство в рекламе</t>
         </is>
       </c>
       <c r="Z14" s="10" t="n"/>
@@ -1857,7 +1949,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Кладовщик на вахте — Яндекс Маркет</t>
+          <t>Кладовщик Яндекс Маркета</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1882,7 +1974,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>vahta</t>
+          <t>flex,full</t>
         </is>
       </c>
       <c r="J15" s="3" t="n">
@@ -1891,13 +1983,17 @@
       <c r="K15" s="3" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Работа на складе вахтой: жильё и питание обычно предоставляются.</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr"/>
+          <t>Работа на складе: оплачиваемая стажировка 3 дня, дальше гибкое расписание смен.</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Стажировка 3 дня ≈ 10 000 ₽, доход до 5 500 ₽ за смену, выплаты еженедельно на карту.</t>
+        </is>
+      </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>Паспорт</t>
+          <t>Паспорт РФ</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -1909,7 +2005,7 @@
         <v>14</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15" s="5" t="n">
         <v>14850</v>
@@ -1938,7 +2034,7 @@
       </c>
       <c r="Y15" s="3" t="inlineStr">
         <is>
-          <t>Условия вахты, куда ехать, жильё</t>
+          <t>ВЫКЛЮЧЕН: из Telegram разрешены только посты в группах/каналах, бот не указан — спросить менеджера. Екатеринбург в гео есть. Конверсия = трудоустройство + 2 или 5 смен</t>
         </is>
       </c>
       <c r="Z15" s="10" t="n"/>

</xml_diff>

<commit_message>
Record Ekaterinburg geo checks for 2304, 2085, 2501
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015gDLhwgHQJ9auhFtnwdBUw
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -830,7 +830,7 @@
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
-          <t>Есть ли Екатеринбург в гео (раздел «Баннеры»). Конверсия = 5 заказов за 14 дней. Чат-боты разрешены; нельзя крупные TG-каналы 50k+. В рекламе писать «партнёр сервиса», без слов про трудоустройство</t>
+          <t>Екатеринбург в гео есть (проверено в кабинете 09.10.2026). Конверсия = 5 заказов за 14 дней. Чат-боты разрешены; нельзя крупные TG-каналы 50k+. В рекламе писать «партнёр сервиса», без слов про трудоустройство</t>
         </is>
       </c>
       <c r="Z2" s="10" t="n"/>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
-          <t>Есть ли Екатеринбург в гео (раздел «Промоматериалы»). Что считается валидной заявкой. Чат-боты разрешены. В рекламе НЕЛЬЗЯ указывать пол, возраст, гражданство, наличие авто</t>
+          <t>Гео Екатеринбург в кабинете не найдено — включён под допущение; через неделю проверить статусы заявок в Pampadu, при отклонениях по гео выключить. Что считается валидной заявкой. Чат-боты разрешены. В рекламе НЕЛЬЗЯ указывать пол, возраст, гражданство, наличие авто</t>
         </is>
       </c>
       <c r="Z5" s="10" t="n"/>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t>Есть ли Екатеринбург в гео (раздел «Баннеры»). Чат-боты разрешены</t>
+          <t>Екатеринбург в гео есть (проверено в кабинете 09.10.2026). Чат-боты разрешены</t>
         </is>
       </c>
       <c r="Z8" s="8" t="inlineStr">

</xml_diff>